<commit_message>
Update generated dependency plots and tables
Regenerate dependency visualizations and spreadsheets (PNG and XLSX) under output/graficos_dependencia. Updates cover comunal and regional plots for multiple regions across years 2018–2024 (e.g. Antofagasta, Araucanía, Arica y Parinacota, Atacama, Biobío, Coquimbo, Los Lagos, Los Ríos, Magallanes, Maule, Metropolitana, Ñuble, O'Higgins, Tarapacá, Valparaíso, Aysén). These are regenerated output files (no source code changes).
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_cobertura/plot_regional_cobertura_2023_tarapaca.xlsx
+++ b/output/graficos_regionales_cobertura/plot_regional_cobertura_2023_tarapaca.xlsx
@@ -418,7 +418,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>Desagregación 1</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -491,13 +491,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>Desagregación 1</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -529,17 +529,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Tamarugal</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>31000</v>
+      </c>
+      <c r="D2">
+        <v>30711</v>
+      </c>
+      <c r="E2">
+        <v>100.9410309009801</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tarapacá</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Iquique</t>
         </is>
       </c>
-      <c r="C2">
-        <v>381064</v>
-      </c>
-      <c r="D2">
-        <v>401588</v>
-      </c>
-      <c r="E2">
-        <v>94.8892895206032</v>
+      <c r="C3">
+        <v>350064</v>
+      </c>
+      <c r="D3">
+        <v>370877</v>
+      </c>
+      <c r="E3">
+        <v>94.3881664271443</v>
       </c>
     </row>
   </sheetData>
@@ -555,7 +576,7 @@
     <row r="1" s="1" customFormat="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>Desagregación 1</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">

</xml_diff>